<commit_message>
Ensure fully deterministic ZIP output across net48 and net10.0
  - Replace framework ZipArchive writing with raw ZipStorer to guarantee
    compression method 0 (Stored) on all frameworks (net48 ignores
    CompressionLevel.NoCompression)
  - Write raw zlib stored blocks in PngNormalizer to avoid DEFLATE
    differences between framework ZLibStream implementations
  - Sort ZIP entries by name using ordinal comparison
  - Sort [Content_Types].xml elements deterministically (ContentTypesPatcher)
  - Renumber all relationship IDs in .rels files to DeterministicId{n} and
    remap corresponding r:id references in content XML
  - Add verification tests for stored entries, deterministic relationship
    IDs, and sorted content types
</commit_message>
<xml_diff>
--- a/src/Tests/Tests.AbsPath.Net.verified.xlsx
+++ b/src/Tests/Tests.AbsPath.Net.verified.xlsx
@@ -7,8 +7,8 @@
     <workbookView xWindow="4290" yWindow="4290" windowWidth="38700" windowHeight="15345" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId3"/>
-    <sheet name="Evaluation Warning" sheetId="2" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="DeterministicId5"/>
+    <sheet name="Evaluation Warning" sheetId="2" r:id="DeterministicId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029"/>

</xml_diff>